<commit_message>
fix(voyages): éviter la relecture systématique des anciens documents
La publication reparcourait tous les voyages après chaque scan,
multipliant les accès Nextcloud et donnant l’impression d’une boucle
lors des expirations de connexion.

- Réutiliser les fiches inchangées à partir de voyage.json.
- Mettre en cache les sections inchangées des éléments à vérifier.
- Conserver une vérification complète pour contrôler et réparer les exports.
- Prendre en compte l’annulation et limiter les lectures à 30 secondes.
- Afficher la progression et documenter le diagnostic Nextcloud.
- Passer la version à 0.3.32.

Validation : 256 tests réussis, MSI compilé et signé.
Contrôle en lecture seule : 95 voyages sur 109 réutilisables.
</commit_message>
<xml_diff>
--- a/mails/mail_list.xlsx
+++ b/mails/mail_list.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\pyoutlookmailing\mails\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBD994E8-5F9D-4422-A7B2-BB5C9815BBBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D84745B-58E2-4758-8292-5104C9FEC426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="20596" windowHeight="13695" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9966" uniqueCount="3168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10080" uniqueCount="3230">
   <si>
     <t>EmailAptitudeEn</t>
   </si>
@@ -9548,6 +9548,192 @@
   </si>
   <si>
     <t>ALLFR2026</t>
+  </si>
+  <si>
+    <t>MOU2026</t>
+  </si>
+  <si>
+    <t>Eric.THEA@be-ys.com</t>
+  </si>
+  <si>
+    <t>Esther.makaay@signicat.com</t>
+  </si>
+  <si>
+    <t>Franck.Ferrandino@infineon.com</t>
+  </si>
+  <si>
+    <t>Laura.Noye@entrust.com</t>
+  </si>
+  <si>
+    <t>Laurence.PROVOTAL@doxallia.com</t>
+  </si>
+  <si>
+    <t>Laurent.Lafargue@cryptomathic.com</t>
+  </si>
+  <si>
+    <t>Michel.Sahli1@swisscom.com</t>
+  </si>
+  <si>
+    <t>Okamoto-R4@mail.dnp.co.jp</t>
+  </si>
+  <si>
+    <t>Patrick.Tabourin@entrust.com</t>
+  </si>
+  <si>
+    <t>Raphael.Guye@swisscom.com</t>
+  </si>
+  <si>
+    <t>Robert.Musick@swisscom.com</t>
+  </si>
+  <si>
+    <t>Roman.Zoun@swisscom.com</t>
+  </si>
+  <si>
+    <t>Sharanya.Thakur@entrust.com</t>
+  </si>
+  <si>
+    <t>Tudor.Stoicescu@entrust.com</t>
+  </si>
+  <si>
+    <t>a.rombi@certeurope.fr</t>
+  </si>
+  <si>
+    <t>aandrieu@icover-services.com</t>
+  </si>
+  <si>
+    <t>anthony.bouyer@digitemis.com</t>
+  </si>
+  <si>
+    <t>antoine.schweitzer-chaput@eviden.com</t>
+  </si>
+  <si>
+    <t>b.dupart@stid.com</t>
+  </si>
+  <si>
+    <t>baris.gumustas@idnow.io</t>
+  </si>
+  <si>
+    <t>benjamin.vignau@coeur-net.fr</t>
+  </si>
+  <si>
+    <t>bruno.bouvier@worldline.com</t>
+  </si>
+  <si>
+    <t>bruno.castanier@univ-angers.fr</t>
+  </si>
+  <si>
+    <t>bruno.urquiza@magellan-partners.eu</t>
+  </si>
+  <si>
+    <t>cecilia.martinez@signicat.com</t>
+  </si>
+  <si>
+    <t>christophe.peix@paragon-id.com</t>
+  </si>
+  <si>
+    <t>contact@synap6.fr</t>
+  </si>
+  <si>
+    <t>contact@xelians.fr</t>
+  </si>
+  <si>
+    <t>david.coridun@goodflag.com</t>
+  </si>
+  <si>
+    <t>ellen.martin@angerstechnopole.com</t>
+  </si>
+  <si>
+    <t>emmanuel.lichou@angerstechnopole.com</t>
+  </si>
+  <si>
+    <t>eric.bultel@st.com</t>
+  </si>
+  <si>
+    <t>fl.doyez@fntc-numerique.com</t>
+  </si>
+  <si>
+    <t>florent.perreux@clever-cloud.com</t>
+  </si>
+  <si>
+    <t>florian@datasure.eu</t>
+  </si>
+  <si>
+    <t>gerard.martinez@aktantis.com</t>
+  </si>
+  <si>
+    <t>gilles.barre@aigcev.org</t>
+  </si>
+  <si>
+    <t>government.affairs@incode.com</t>
+  </si>
+  <si>
+    <t>info@ver.id</t>
+  </si>
+  <si>
+    <t>jbe@evertrust.fr</t>
+  </si>
+  <si>
+    <t>jean-luc@trustandcie.fr</t>
+  </si>
+  <si>
+    <t>jerome.frou@linxens.com</t>
+  </si>
+  <si>
+    <t>ludovic.decarcouet@digitemis.com</t>
+  </si>
+  <si>
+    <t>m.depassorio@groupeonepoint.com</t>
+  </si>
+  <si>
+    <t>m.wajnglas@spac-alliance.org</t>
+  </si>
+  <si>
+    <t>marc.lavorel@id3.eu</t>
+  </si>
+  <si>
+    <t>marc.piepers@coppernic.com</t>
+  </si>
+  <si>
+    <t>michel.hatiez@magellan-consulting.eu</t>
+  </si>
+  <si>
+    <t>nicolas.million-picalion@airweb.fr</t>
+  </si>
+  <si>
+    <t>olivier.zemerli@ascertia.com</t>
+  </si>
+  <si>
+    <t>p.courpron@groupeonepoint.com</t>
+  </si>
+  <si>
+    <t>patrice.polidori@digitech.fr</t>
+  </si>
+  <si>
+    <t>philippe.luc@anozrway.com</t>
+  </si>
+  <si>
+    <t>pol.roland-billecart@tnpconsultants.com</t>
+  </si>
+  <si>
+    <t>quentin.adam@clever-cloud.com</t>
+  </si>
+  <si>
+    <t>s.hamdoune@selp.fr</t>
+  </si>
+  <si>
+    <t>swan@shareid.ai</t>
+  </si>
+  <si>
+    <t>thomasdewilde@sofie.fr</t>
+  </si>
+  <si>
+    <t>yacine.tamoudi@kereval.com</t>
+  </si>
+  <si>
+    <t>yassine.mountacif@unissey.com</t>
+  </si>
+  <si>
+    <t>zoe.bonald@famoco.com</t>
   </si>
 </sst>
 </file>
@@ -12039,7 +12225,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AV1287"/>
+  <dimension ref="A1:AW1287"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="27.796875" customWidth="1"/>
@@ -12087,7 +12273,7 @@
     <col min="49" max="49" width="34.9296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>1605</v>
       </c>
@@ -12223,8 +12409,11 @@
       <c r="AV1" s="2" t="s">
         <v>3167</v>
       </c>
-    </row>
-    <row r="2" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW1" s="2" t="s">
+        <v>3168</v>
+      </c>
+    </row>
+    <row r="2" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>1310</v>
       </c>
@@ -12360,8 +12549,11 @@
       <c r="AV2" t="s">
         <v>2357</v>
       </c>
-    </row>
-    <row r="3" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW2" t="s">
+        <v>3169</v>
+      </c>
+    </row>
+    <row r="3" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>17</v>
       </c>
@@ -12492,8 +12684,11 @@
       <c r="AV3" t="s">
         <v>2365</v>
       </c>
-    </row>
-    <row r="4" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW3" t="s">
+        <v>3170</v>
+      </c>
+    </row>
+    <row r="4" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>216</v>
       </c>
@@ -12617,8 +12812,11 @@
       <c r="AV4" t="s">
         <v>2368</v>
       </c>
-    </row>
-    <row r="5" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW4" t="s">
+        <v>3171</v>
+      </c>
+    </row>
+    <row r="5" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>1589</v>
       </c>
@@ -12736,8 +12934,11 @@
       <c r="AV5" t="s">
         <v>2374</v>
       </c>
-    </row>
-    <row r="6" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW5" t="s">
+        <v>3172</v>
+      </c>
+    </row>
+    <row r="6" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>235</v>
       </c>
@@ -12855,8 +13056,11 @@
       <c r="AV6" t="s">
         <v>2375</v>
       </c>
-    </row>
-    <row r="7" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW6" t="s">
+        <v>3173</v>
+      </c>
+    </row>
+    <row r="7" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>1290</v>
       </c>
@@ -12974,8 +13178,11 @@
       <c r="AV7" t="s">
         <v>1617</v>
       </c>
-    </row>
-    <row r="8" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW7" t="s">
+        <v>3174</v>
+      </c>
+    </row>
+    <row r="8" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>1353</v>
       </c>
@@ -13090,8 +13297,11 @@
       <c r="AV8" t="s">
         <v>2390</v>
       </c>
-    </row>
-    <row r="9" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW8" t="s">
+        <v>3175</v>
+      </c>
+    </row>
+    <row r="9" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>1276</v>
       </c>
@@ -13203,8 +13413,11 @@
       <c r="AV9" t="s">
         <v>2391</v>
       </c>
-    </row>
-    <row r="10" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW9" t="s">
+        <v>3176</v>
+      </c>
+    </row>
+    <row r="10" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>217</v>
       </c>
@@ -13316,8 +13529,11 @@
       <c r="AV10" t="s">
         <v>2407</v>
       </c>
-    </row>
-    <row r="11" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW10" t="s">
+        <v>3177</v>
+      </c>
+    </row>
+    <row r="11" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>1292</v>
       </c>
@@ -13429,8 +13645,11 @@
       <c r="AV11" t="s">
         <v>1844</v>
       </c>
-    </row>
-    <row r="12" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW11" t="s">
+        <v>3178</v>
+      </c>
+    </row>
+    <row r="12" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>236</v>
       </c>
@@ -13542,8 +13761,11 @@
       <c r="AV12" t="s">
         <v>489</v>
       </c>
-    </row>
-    <row r="13" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW12" t="s">
+        <v>3179</v>
+      </c>
+    </row>
+    <row r="13" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -13655,8 +13877,11 @@
       <c r="AV13" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="14" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW13" t="s">
+        <v>3180</v>
+      </c>
+    </row>
+    <row r="14" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>8</v>
       </c>
@@ -13768,8 +13993,11 @@
       <c r="AV14" t="s">
         <v>2441</v>
       </c>
-    </row>
-    <row r="15" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW14" t="s">
+        <v>3181</v>
+      </c>
+    </row>
+    <row r="15" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>1351</v>
       </c>
@@ -13881,8 +14109,11 @@
       <c r="AV15" t="s">
         <v>2453</v>
       </c>
-    </row>
-    <row r="16" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW15" t="s">
+        <v>3182</v>
+      </c>
+    </row>
+    <row r="16" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>218</v>
       </c>
@@ -13991,8 +14222,11 @@
       <c r="AV16" t="s">
         <v>1236</v>
       </c>
-    </row>
-    <row r="17" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW16" t="s">
+        <v>3183</v>
+      </c>
+    </row>
+    <row r="17" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>207</v>
       </c>
@@ -14098,8 +14332,11 @@
       <c r="AV17" t="s">
         <v>2463</v>
       </c>
-    </row>
-    <row r="18" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW17" t="s">
+        <v>3184</v>
+      </c>
+    </row>
+    <row r="18" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>1311</v>
       </c>
@@ -14205,8 +14442,11 @@
       <c r="AV18" t="s">
         <v>531</v>
       </c>
-    </row>
-    <row r="19" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW18" t="s">
+        <v>2370</v>
+      </c>
+    </row>
+    <row r="19" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>1288</v>
       </c>
@@ -14312,8 +14552,11 @@
       <c r="AV19" t="s">
         <v>2478</v>
       </c>
-    </row>
-    <row r="20" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW19" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="20" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>242</v>
       </c>
@@ -14419,8 +14662,11 @@
       <c r="AV20" t="s">
         <v>2481</v>
       </c>
-    </row>
-    <row r="21" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW20" t="s">
+        <v>1616</v>
+      </c>
+    </row>
+    <row r="21" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>222</v>
       </c>
@@ -14526,8 +14772,11 @@
       <c r="AV21" t="s">
         <v>2489</v>
       </c>
-    </row>
-    <row r="22" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW21" t="s">
+        <v>2244</v>
+      </c>
+    </row>
+    <row r="22" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>18</v>
       </c>
@@ -14633,8 +14882,11 @@
       <c r="AV22" t="s">
         <v>2490</v>
       </c>
-    </row>
-    <row r="23" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW22" t="s">
+        <v>2389</v>
+      </c>
+    </row>
+    <row r="23" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>1343</v>
       </c>
@@ -14740,8 +14992,11 @@
       <c r="AV23" t="s">
         <v>2498</v>
       </c>
-    </row>
-    <row r="24" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW23" t="s">
+        <v>1521</v>
+      </c>
+    </row>
+    <row r="24" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>295</v>
       </c>
@@ -14841,8 +15096,11 @@
       <c r="AV24" t="s">
         <v>2500</v>
       </c>
-    </row>
-    <row r="25" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW24" t="s">
+        <v>3185</v>
+      </c>
+    </row>
+    <row r="25" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>1590</v>
       </c>
@@ -14942,8 +15200,11 @@
       <c r="AV25" t="s">
         <v>2501</v>
       </c>
-    </row>
-    <row r="26" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW25" t="s">
+        <v>3186</v>
+      </c>
+    </row>
+    <row r="26" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>177</v>
       </c>
@@ -15043,8 +15304,11 @@
       <c r="AV26" t="s">
         <v>2505</v>
       </c>
-    </row>
-    <row r="27" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW26" t="s">
+        <v>1420</v>
+      </c>
+    </row>
+    <row r="27" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>228</v>
       </c>
@@ -15144,8 +15408,11 @@
       <c r="AV27" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="28" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW27" t="s">
+        <v>1622</v>
+      </c>
+    </row>
+    <row r="28" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>1204</v>
       </c>
@@ -15245,8 +15512,11 @@
       <c r="AV28" t="s">
         <v>2509</v>
       </c>
-    </row>
-    <row r="29" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW28" t="s">
+        <v>1522</v>
+      </c>
+    </row>
+    <row r="29" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>1591</v>
       </c>
@@ -15346,8 +15616,11 @@
       <c r="AV29" t="s">
         <v>2514</v>
       </c>
-    </row>
-    <row r="30" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW29" t="s">
+        <v>2438</v>
+      </c>
+    </row>
+    <row r="30" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>227</v>
       </c>
@@ -15447,8 +15720,11 @@
       <c r="AV30" t="s">
         <v>2523</v>
       </c>
-    </row>
-    <row r="31" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW30" t="s">
+        <v>3187</v>
+      </c>
+    </row>
+    <row r="31" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>1592</v>
       </c>
@@ -15548,8 +15824,11 @@
       <c r="AV31" t="s">
         <v>2526</v>
       </c>
-    </row>
-    <row r="32" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW31" t="s">
+        <v>3188</v>
+      </c>
+    </row>
+    <row r="32" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>181</v>
       </c>
@@ -15649,8 +15928,11 @@
       <c r="AV32" t="s">
         <v>2535</v>
       </c>
-    </row>
-    <row r="33" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW32" t="s">
+        <v>3189</v>
+      </c>
+    </row>
+    <row r="33" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>1593</v>
       </c>
@@ -15750,8 +16032,11 @@
       <c r="AV33" t="s">
         <v>1220</v>
       </c>
-    </row>
-    <row r="34" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW33" t="s">
+        <v>1229</v>
+      </c>
+    </row>
+    <row r="34" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>1594</v>
       </c>
@@ -15851,8 +16136,11 @@
       <c r="AV34" t="s">
         <v>2544</v>
       </c>
-    </row>
-    <row r="35" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW34" t="s">
+        <v>1607</v>
+      </c>
+    </row>
+    <row r="35" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>1595</v>
       </c>
@@ -15952,8 +16240,11 @@
       <c r="AV35" t="s">
         <v>2550</v>
       </c>
-    </row>
-    <row r="36" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW35" t="s">
+        <v>3190</v>
+      </c>
+    </row>
+    <row r="36" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
         <v>170</v>
       </c>
@@ -16053,8 +16344,11 @@
       <c r="AV36" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="37" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW36" t="s">
+        <v>3191</v>
+      </c>
+    </row>
+    <row r="37" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>1207</v>
       </c>
@@ -16154,8 +16448,11 @@
       <c r="AV37" t="s">
         <v>2586</v>
       </c>
-    </row>
-    <row r="38" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW37" t="s">
+        <v>3192</v>
+      </c>
+    </row>
+    <row r="38" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>199</v>
       </c>
@@ -16255,8 +16552,11 @@
       <c r="AV38" t="s">
         <v>2590</v>
       </c>
-    </row>
-    <row r="39" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW38" t="s">
+        <v>1378</v>
+      </c>
+    </row>
+    <row r="39" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>53</v>
       </c>
@@ -16356,8 +16656,11 @@
       <c r="AV39" t="s">
         <v>2593</v>
       </c>
-    </row>
-    <row r="40" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW39" t="s">
+        <v>3193</v>
+      </c>
+    </row>
+    <row r="40" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>224</v>
       </c>
@@ -16457,8 +16760,11 @@
       <c r="AV40" t="s">
         <v>2602</v>
       </c>
-    </row>
-    <row r="41" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW40" t="s">
+        <v>3194</v>
+      </c>
+    </row>
+    <row r="41" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>1201</v>
       </c>
@@ -16558,8 +16864,11 @@
       <c r="AV41" t="s">
         <v>2603</v>
       </c>
-    </row>
-    <row r="42" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW41" t="s">
+        <v>1305</v>
+      </c>
+    </row>
+    <row r="42" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>11</v>
       </c>
@@ -16659,8 +16968,11 @@
       <c r="AV42" t="s">
         <v>474</v>
       </c>
-    </row>
-    <row r="43" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW42" t="s">
+        <v>3195</v>
+      </c>
+    </row>
+    <row r="43" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>1596</v>
       </c>
@@ -16760,8 +17072,11 @@
       <c r="AV43" t="s">
         <v>2618</v>
       </c>
-    </row>
-    <row r="44" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW43" t="s">
+        <v>3196</v>
+      </c>
+    </row>
+    <row r="44" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>1338</v>
       </c>
@@ -16861,8 +17176,11 @@
       <c r="AV44" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="45" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW44" t="s">
+        <v>2529</v>
+      </c>
+    </row>
+    <row r="45" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>229</v>
       </c>
@@ -16959,8 +17277,11 @@
       <c r="AV45" t="s">
         <v>2620</v>
       </c>
-    </row>
-    <row r="46" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW45" t="s">
+        <v>3197</v>
+      </c>
+    </row>
+    <row r="46" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>1331</v>
       </c>
@@ -17057,8 +17378,11 @@
       <c r="AV46" t="s">
         <v>529</v>
       </c>
-    </row>
-    <row r="47" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW46" t="s">
+        <v>3198</v>
+      </c>
+    </row>
+    <row r="47" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
         <v>30</v>
       </c>
@@ -17155,8 +17479,11 @@
       <c r="AV47" t="s">
         <v>47</v>
       </c>
-    </row>
-    <row r="48" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW47" t="s">
+        <v>3199</v>
+      </c>
+    </row>
+    <row r="48" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>31</v>
       </c>
@@ -17253,8 +17580,11 @@
       <c r="AV48" t="s">
         <v>1224</v>
       </c>
-    </row>
-    <row r="49" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW48" t="s">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="49" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>223</v>
       </c>
@@ -17348,8 +17678,11 @@
       <c r="AV49" t="s">
         <v>2623</v>
       </c>
-    </row>
-    <row r="50" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW49" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="50" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>16</v>
       </c>
@@ -17443,8 +17776,11 @@
       <c r="AV50" t="s">
         <v>2624</v>
       </c>
-    </row>
-    <row r="51" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW50" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="51" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>1309</v>
       </c>
@@ -17535,8 +17871,11 @@
       <c r="AV51" t="s">
         <v>2630</v>
       </c>
-    </row>
-    <row r="52" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW51" t="s">
+        <v>3201</v>
+      </c>
+    </row>
+    <row r="52" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>230</v>
       </c>
@@ -17627,8 +17966,11 @@
       <c r="AV52" t="s">
         <v>2634</v>
       </c>
-    </row>
-    <row r="53" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW52" t="s">
+        <v>3202</v>
+      </c>
+    </row>
+    <row r="53" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
         <v>1208</v>
       </c>
@@ -17719,8 +18061,11 @@
       <c r="AV53" t="s">
         <v>1464</v>
       </c>
-    </row>
-    <row r="54" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW53" t="s">
+        <v>3203</v>
+      </c>
+    </row>
+    <row r="54" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
         <v>149</v>
       </c>
@@ -17811,8 +18156,11 @@
       <c r="AV54" t="s">
         <v>2648</v>
       </c>
-    </row>
-    <row r="55" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW54" t="s">
+        <v>1517</v>
+      </c>
+    </row>
+    <row r="55" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>34</v>
       </c>
@@ -17903,8 +18251,11 @@
       <c r="AV55" t="s">
         <v>1614</v>
       </c>
-    </row>
-    <row r="56" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW55" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="56" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
         <v>1321</v>
       </c>
@@ -17995,8 +18346,11 @@
       <c r="AV56" t="s">
         <v>2655</v>
       </c>
-    </row>
-    <row r="57" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW56" t="s">
+        <v>3204</v>
+      </c>
+    </row>
+    <row r="57" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
         <v>270</v>
       </c>
@@ -18087,8 +18441,11 @@
       <c r="AV57" t="s">
         <v>491</v>
       </c>
-    </row>
-    <row r="58" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW57" t="s">
+        <v>3205</v>
+      </c>
+    </row>
+    <row r="58" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
         <v>1597</v>
       </c>
@@ -18176,8 +18533,11 @@
       <c r="AV58" t="s">
         <v>2656</v>
       </c>
-    </row>
-    <row r="59" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW58" t="s">
+        <v>3206</v>
+      </c>
+    </row>
+    <row r="59" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
         <v>115</v>
       </c>
@@ -18265,8 +18625,11 @@
       <c r="AV59" t="s">
         <v>2657</v>
       </c>
-    </row>
-    <row r="60" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW59" t="s">
+        <v>1849</v>
+      </c>
+    </row>
+    <row r="60" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
         <v>1283</v>
       </c>
@@ -18354,8 +18717,11 @@
       <c r="AV60" t="s">
         <v>2658</v>
       </c>
-    </row>
-    <row r="61" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW60" t="s">
+        <v>2658</v>
+      </c>
+    </row>
+    <row r="61" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
         <v>62</v>
       </c>
@@ -18443,8 +18809,11 @@
       <c r="AV61" t="s">
         <v>2665</v>
       </c>
-    </row>
-    <row r="62" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW61" t="s">
+        <v>2669</v>
+      </c>
+    </row>
+    <row r="62" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
         <v>146</v>
       </c>
@@ -18532,8 +18901,11 @@
       <c r="AV62" t="s">
         <v>2060</v>
       </c>
-    </row>
-    <row r="63" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW62" t="s">
+        <v>1361</v>
+      </c>
+    </row>
+    <row r="63" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
         <v>1313</v>
       </c>
@@ -18621,8 +18993,11 @@
       <c r="AV63" t="s">
         <v>2671</v>
       </c>
-    </row>
-    <row r="64" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW63" t="s">
+        <v>3207</v>
+      </c>
+    </row>
+    <row r="64" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
         <v>1350</v>
       </c>
@@ -18710,8 +19085,11 @@
       <c r="AV64" t="s">
         <v>2067</v>
       </c>
-    </row>
-    <row r="65" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW64" t="s">
+        <v>3208</v>
+      </c>
+    </row>
+    <row r="65" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
         <v>158</v>
       </c>
@@ -18799,8 +19177,11 @@
       <c r="AV65" t="s">
         <v>2705</v>
       </c>
-    </row>
-    <row r="66" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW65" t="s">
+        <v>3209</v>
+      </c>
+    </row>
+    <row r="66" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
         <v>42</v>
       </c>
@@ -18888,8 +19269,11 @@
       <c r="AV66" t="s">
         <v>2720</v>
       </c>
-    </row>
-    <row r="67" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW66" t="s">
+        <v>2736</v>
+      </c>
+    </row>
+    <row r="67" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
         <v>233</v>
       </c>
@@ -18974,8 +19358,11 @@
       <c r="AV67" t="s">
         <v>2728</v>
       </c>
-    </row>
-    <row r="68" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW67" t="s">
+        <v>3210</v>
+      </c>
+    </row>
+    <row r="68" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
         <v>85</v>
       </c>
@@ -19060,8 +19447,11 @@
       <c r="AV68" t="s">
         <v>1244</v>
       </c>
-    </row>
-    <row r="69" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW68" t="s">
+        <v>2282</v>
+      </c>
+    </row>
+    <row r="69" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
         <v>12</v>
       </c>
@@ -19146,8 +19536,11 @@
       <c r="AV69" t="s">
         <v>2733</v>
       </c>
-    </row>
-    <row r="70" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW69" t="s">
+        <v>1831</v>
+      </c>
+    </row>
+    <row r="70" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
         <v>489</v>
       </c>
@@ -19232,8 +19625,11 @@
       <c r="AV70" t="s">
         <v>2734</v>
       </c>
-    </row>
-    <row r="71" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW70" t="s">
+        <v>1372</v>
+      </c>
+    </row>
+    <row r="71" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
         <v>103</v>
       </c>
@@ -19318,8 +19714,11 @@
       <c r="AV71" t="s">
         <v>1937</v>
       </c>
-    </row>
-    <row r="72" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW71" t="s">
+        <v>2795</v>
+      </c>
+    </row>
+    <row r="72" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
         <v>313</v>
       </c>
@@ -19404,8 +19803,11 @@
       <c r="AV72" t="s">
         <v>2735</v>
       </c>
-    </row>
-    <row r="73" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW72" t="s">
+        <v>2804</v>
+      </c>
+    </row>
+    <row r="73" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
         <v>157</v>
       </c>
@@ -19490,8 +19892,11 @@
       <c r="AV73" t="s">
         <v>2742</v>
       </c>
-    </row>
-    <row r="74" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW73" t="s">
+        <v>3211</v>
+      </c>
+    </row>
+    <row r="74" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
         <v>40</v>
       </c>
@@ -19576,8 +19981,11 @@
       <c r="AV74" t="s">
         <v>1381</v>
       </c>
-    </row>
-    <row r="75" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW74" t="s">
+        <v>3212</v>
+      </c>
+    </row>
+    <row r="75" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
         <v>124</v>
       </c>
@@ -19662,8 +20070,11 @@
       <c r="AV75" t="s">
         <v>2756</v>
       </c>
-    </row>
-    <row r="76" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW75" t="s">
+        <v>3213</v>
+      </c>
+    </row>
+    <row r="76" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
         <v>1438</v>
       </c>
@@ -19748,8 +20159,11 @@
       <c r="AV76" t="s">
         <v>2766</v>
       </c>
-    </row>
-    <row r="77" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW76" t="s">
+        <v>2821</v>
+      </c>
+    </row>
+    <row r="77" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
         <v>112</v>
       </c>
@@ -19834,8 +20248,11 @@
       <c r="AV77" t="s">
         <v>1640</v>
       </c>
-    </row>
-    <row r="78" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW77" t="s">
+        <v>3214</v>
+      </c>
+    </row>
+    <row r="78" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
         <v>99</v>
       </c>
@@ -19917,8 +20334,11 @@
       <c r="AV78" t="s">
         <v>2776</v>
       </c>
-    </row>
-    <row r="79" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW78" t="s">
+        <v>3215</v>
+      </c>
+    </row>
+    <row r="79" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
         <v>652</v>
       </c>
@@ -20000,8 +20420,11 @@
       <c r="AV79" t="s">
         <v>2779</v>
       </c>
-    </row>
-    <row r="80" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW79" t="s">
+        <v>2295</v>
+      </c>
+    </row>
+    <row r="80" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
         <v>231</v>
       </c>
@@ -20083,8 +20506,11 @@
       <c r="AV80" t="s">
         <v>510</v>
       </c>
-    </row>
-    <row r="81" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW80" t="s">
+        <v>1813</v>
+      </c>
+    </row>
+    <row r="81" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
         <v>87</v>
       </c>
@@ -20166,8 +20592,11 @@
       <c r="AV81" t="s">
         <v>2782</v>
       </c>
-    </row>
-    <row r="82" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW81" t="s">
+        <v>2859</v>
+      </c>
+    </row>
+    <row r="82" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
         <v>142</v>
       </c>
@@ -20249,8 +20678,11 @@
       <c r="AV82" t="s">
         <v>2789</v>
       </c>
-    </row>
-    <row r="83" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW82" t="s">
+        <v>3216</v>
+      </c>
+    </row>
+    <row r="83" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
         <v>201</v>
       </c>
@@ -20332,8 +20764,11 @@
       <c r="AV83" t="s">
         <v>509</v>
       </c>
-    </row>
-    <row r="84" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW83" t="s">
+        <v>2868</v>
+      </c>
+    </row>
+    <row r="84" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
         <v>220</v>
       </c>
@@ -20415,8 +20850,11 @@
       <c r="AV84" t="s">
         <v>2796</v>
       </c>
-    </row>
-    <row r="85" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW84" t="s">
+        <v>3217</v>
+      </c>
+    </row>
+    <row r="85" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
         <v>150</v>
       </c>
@@ -20498,8 +20936,11 @@
       <c r="AV85" t="s">
         <v>381</v>
       </c>
-    </row>
-    <row r="86" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW85" t="s">
+        <v>1518</v>
+      </c>
+    </row>
+    <row r="86" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
         <v>1319</v>
       </c>
@@ -20581,8 +21022,11 @@
       <c r="AV86" t="s">
         <v>1857</v>
       </c>
-    </row>
-    <row r="87" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW86" t="s">
+        <v>2921</v>
+      </c>
+    </row>
+    <row r="87" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
         <v>249</v>
       </c>
@@ -20664,8 +21108,11 @@
       <c r="AV87" t="s">
         <v>2799</v>
       </c>
-    </row>
-    <row r="88" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW87" t="s">
+        <v>1230</v>
+      </c>
+    </row>
+    <row r="88" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
         <v>1285</v>
       </c>
@@ -20744,8 +21191,11 @@
       <c r="AV88" t="s">
         <v>2800</v>
       </c>
-    </row>
-    <row r="89" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW88" t="s">
+        <v>3218</v>
+      </c>
+    </row>
+    <row r="89" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
         <v>679</v>
       </c>
@@ -20824,8 +21274,11 @@
       <c r="AV89" t="s">
         <v>2803</v>
       </c>
-    </row>
-    <row r="90" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW89" t="s">
+        <v>3219</v>
+      </c>
+    </row>
+    <row r="90" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
         <v>1280</v>
       </c>
@@ -20904,8 +21357,11 @@
       <c r="AV90" t="s">
         <v>301</v>
       </c>
-    </row>
-    <row r="91" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW90" t="s">
+        <v>2942</v>
+      </c>
+    </row>
+    <row r="91" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
         <v>1265</v>
       </c>
@@ -20982,8 +21438,11 @@
       <c r="AV91" t="s">
         <v>2823</v>
       </c>
-    </row>
-    <row r="92" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW91" t="s">
+        <v>3220</v>
+      </c>
+    </row>
+    <row r="92" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
         <v>1305</v>
       </c>
@@ -21059,8 +21518,11 @@
       <c r="AV92" t="s">
         <v>2824</v>
       </c>
-    </row>
-    <row r="93" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW92" t="s">
+        <v>3221</v>
+      </c>
+    </row>
+    <row r="93" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
         <v>96</v>
       </c>
@@ -21136,8 +21598,11 @@
       <c r="AV93" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="94" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW93" t="s">
+        <v>3222</v>
+      </c>
+    </row>
+    <row r="94" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
         <v>116</v>
       </c>
@@ -21213,8 +21678,11 @@
       <c r="AV94" t="s">
         <v>2829</v>
       </c>
-    </row>
-    <row r="95" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW94" t="s">
+        <v>3223</v>
+      </c>
+    </row>
+    <row r="95" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
         <v>1429</v>
       </c>
@@ -21290,8 +21758,11 @@
       <c r="AV95" t="s">
         <v>1240</v>
       </c>
-    </row>
-    <row r="96" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW95" t="s">
+        <v>2997</v>
+      </c>
+    </row>
+    <row r="96" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
         <v>1275</v>
       </c>
@@ -21364,8 +21835,11 @@
       <c r="AV96" t="s">
         <v>1221</v>
       </c>
-    </row>
-    <row r="97" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW96" t="s">
+        <v>3002</v>
+      </c>
+    </row>
+    <row r="97" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
         <v>1598</v>
       </c>
@@ -21438,8 +21912,11 @@
       <c r="AV97" t="s">
         <v>304</v>
       </c>
-    </row>
-    <row r="98" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW97" t="s">
+        <v>1983</v>
+      </c>
+    </row>
+    <row r="98" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
         <v>140</v>
       </c>
@@ -21512,8 +21989,11 @@
       <c r="AV98" t="s">
         <v>522</v>
       </c>
-    </row>
-    <row r="99" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW98" t="s">
+        <v>3015</v>
+      </c>
+    </row>
+    <row r="99" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
         <v>243</v>
       </c>
@@ -21586,8 +22066,11 @@
       <c r="AV99" t="s">
         <v>2832</v>
       </c>
-    </row>
-    <row r="100" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW99" t="s">
+        <v>3224</v>
+      </c>
+    </row>
+    <row r="100" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
         <v>98</v>
       </c>
@@ -21660,8 +22143,11 @@
       <c r="AV100" t="s">
         <v>2844</v>
       </c>
-    </row>
-    <row r="101" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW100" t="s">
+        <v>3023</v>
+      </c>
+    </row>
+    <row r="101" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
         <v>240</v>
       </c>
@@ -21734,8 +22220,11 @@
       <c r="AV101" t="s">
         <v>2847</v>
       </c>
-    </row>
-    <row r="102" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW101" t="s">
+        <v>1527</v>
+      </c>
+    </row>
+    <row r="102" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A102" t="s">
         <v>127</v>
       </c>
@@ -21805,8 +22294,11 @@
       <c r="AV102" t="s">
         <v>1834</v>
       </c>
-    </row>
-    <row r="103" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW102" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="103" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A103" t="s">
         <v>1320</v>
       </c>
@@ -21876,8 +22368,11 @@
       <c r="AV103" t="s">
         <v>2863</v>
       </c>
-    </row>
-    <row r="104" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW103" t="s">
+        <v>3069</v>
+      </c>
+    </row>
+    <row r="104" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A104" t="s">
         <v>36</v>
       </c>
@@ -21947,8 +22442,11 @@
       <c r="AV104" t="s">
         <v>2870</v>
       </c>
-    </row>
-    <row r="105" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW104" t="s">
+        <v>3077</v>
+      </c>
+    </row>
+    <row r="105" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A105" t="s">
         <v>244</v>
       </c>
@@ -22018,8 +22516,11 @@
       <c r="AV105" t="s">
         <v>2871</v>
       </c>
-    </row>
-    <row r="106" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW105" t="s">
+        <v>3225</v>
+      </c>
+    </row>
+    <row r="106" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A106" t="s">
         <v>178</v>
       </c>
@@ -22089,8 +22590,11 @@
       <c r="AV106" t="s">
         <v>2884</v>
       </c>
-    </row>
-    <row r="107" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW106" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="107" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A107" t="s">
         <v>162</v>
       </c>
@@ -22157,8 +22661,11 @@
       <c r="AV107" t="s">
         <v>2887</v>
       </c>
-    </row>
-    <row r="108" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW107" t="s">
+        <v>3102</v>
+      </c>
+    </row>
+    <row r="108" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A108" t="s">
         <v>1200</v>
       </c>
@@ -22225,8 +22732,11 @@
       <c r="AV108" t="s">
         <v>2888</v>
       </c>
-    </row>
-    <row r="109" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW108" t="s">
+        <v>1227</v>
+      </c>
+    </row>
+    <row r="109" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A109" t="s">
         <v>186</v>
       </c>
@@ -22293,8 +22803,11 @@
       <c r="AV109" t="s">
         <v>2890</v>
       </c>
-    </row>
-    <row r="110" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW109" t="s">
+        <v>3226</v>
+      </c>
+    </row>
+    <row r="110" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A110" t="s">
         <v>1314</v>
       </c>
@@ -22358,8 +22871,11 @@
       <c r="AV110" t="s">
         <v>2893</v>
       </c>
-    </row>
-    <row r="111" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW110" t="s">
+        <v>3227</v>
+      </c>
+    </row>
+    <row r="111" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A111" t="s">
         <v>136</v>
       </c>
@@ -22423,8 +22939,11 @@
       <c r="AV111" t="s">
         <v>1488</v>
       </c>
-    </row>
-    <row r="112" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW111" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="112" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A112" t="s">
         <v>1281</v>
       </c>
@@ -22488,8 +23007,11 @@
       <c r="AV112" t="s">
         <v>530</v>
       </c>
-    </row>
-    <row r="113" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW112" t="s">
+        <v>3228</v>
+      </c>
+    </row>
+    <row r="113" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A113" t="s">
         <v>1430</v>
       </c>
@@ -22550,8 +23072,11 @@
       <c r="AV113" t="s">
         <v>2902</v>
       </c>
-    </row>
-    <row r="114" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW113" t="s">
+        <v>1358</v>
+      </c>
+    </row>
+    <row r="114" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A114" t="s">
         <v>108</v>
       </c>
@@ -22612,8 +23137,11 @@
       <c r="AV114" t="s">
         <v>1835</v>
       </c>
-    </row>
-    <row r="115" spans="1:48" x14ac:dyDescent="0.45">
+      <c r="AW114" t="s">
+        <v>3229</v>
+      </c>
+    </row>
+    <row r="115" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A115" t="s">
         <v>100</v>
       </c>
@@ -22675,7 +23203,7 @@
         <v>2135</v>
       </c>
     </row>
-    <row r="116" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A116" t="s">
         <v>200</v>
       </c>
@@ -22737,7 +23265,7 @@
         <v>2940</v>
       </c>
     </row>
-    <row r="117" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A117" t="s">
         <v>1318</v>
       </c>
@@ -22799,7 +23327,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="118" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A118" t="s">
         <v>166</v>
       </c>
@@ -22861,7 +23389,7 @@
         <v>2943</v>
       </c>
     </row>
-    <row r="119" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="119" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A119" t="s">
         <v>749</v>
       </c>
@@ -22923,7 +23451,7 @@
         <v>2944</v>
       </c>
     </row>
-    <row r="120" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A120" t="s">
         <v>1300</v>
       </c>
@@ -22985,7 +23513,7 @@
         <v>2946</v>
       </c>
     </row>
-    <row r="121" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A121" t="s">
         <v>160</v>
       </c>
@@ -23047,7 +23575,7 @@
         <v>2948</v>
       </c>
     </row>
-    <row r="122" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A122" t="s">
         <v>1460</v>
       </c>
@@ -23109,7 +23637,7 @@
         <v>2949</v>
       </c>
     </row>
-    <row r="123" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A123" t="s">
         <v>4</v>
       </c>
@@ -23168,7 +23696,7 @@
         <v>2955</v>
       </c>
     </row>
-    <row r="124" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A124" t="s">
         <v>132</v>
       </c>
@@ -23227,7 +23755,7 @@
         <v>1861</v>
       </c>
     </row>
-    <row r="125" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A125" t="s">
         <v>1431</v>
       </c>
@@ -23286,7 +23814,7 @@
         <v>2960</v>
       </c>
     </row>
-    <row r="126" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="126" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A126" t="s">
         <v>1334</v>
       </c>
@@ -23345,7 +23873,7 @@
         <v>490</v>
       </c>
     </row>
-    <row r="127" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="127" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A127" t="s">
         <v>58</v>
       </c>
@@ -23404,7 +23932,7 @@
         <v>2962</v>
       </c>
     </row>
-    <row r="128" spans="1:48" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:49" x14ac:dyDescent="0.45">
       <c r="A128" t="s">
         <v>20</v>
       </c>

</xml_diff>